<commit_message>
add prepared results for 2021 and 2024
first look to identify main results
</commit_message>
<xml_diff>
--- a/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/01_raw_results/outputs_IAEE_2025_run_2021_no_limits.xlsx
+++ b/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/01_raw_results/outputs_IAEE_2025_run_2021_no_limits.xlsx
@@ -458,14 +458,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>('DE', 'LU')</t>
+          <t>('DZ', 'ES')</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>7673.318317179277</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.06236366036808132</v>
       </c>
     </row>
     <row r="3">
@@ -476,14 +476,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>('DZ', 'ES')</t>
+          <t>('RS', 'BA')</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9138.818317179161</v>
+        <v>6562.7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.07427427589211087</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -494,14 +494,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>('UA', 'MD')</t>
+          <t>('AL', 'IT')</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6993.868709865174</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.07500684468945812</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -512,7 +512,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>('DK', 'DE')</t>
+          <t>('FR', 'ES')</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -530,14 +530,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>('MD', 'RO')</t>
+          <t>('NL', 'BE')</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>5319.754029749992</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.01043134023379438</v>
       </c>
     </row>
     <row r="7">
@@ -548,14 +548,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>('DZ', 'TN')</t>
+          <t>('LT', 'LV')</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>355847.9983900771</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0.856625975737205</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -566,14 +566,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>('DE', 'PL')</t>
+          <t>('AT', 'IT')</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>78271.18871345275</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>0.1864709677509297</v>
       </c>
     </row>
     <row r="9">
@@ -584,14 +584,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>('BE', 'FR')</t>
+          <t>('PL', 'DE')</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>114691.6019731564</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>0.3372945116463543</v>
       </c>
     </row>
     <row r="10">
@@ -602,14 +602,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>('RU', 'LV')</t>
+          <t>('EE', 'LV')</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>33546.970555</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5470804069634703</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -620,14 +620,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>('EE', 'LV')</t>
+          <t>('FI', 'EE')</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>4201.588500000001</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>0.3509271885270984</v>
       </c>
     </row>
     <row r="12">
@@ -638,7 +638,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>('LT', 'LV')</t>
+          <t>('DE', 'BE')</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -656,14 +656,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>('NO', 'NL')</t>
+          <t>('FR', 'BE')</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>123813.4545419723</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0.3520287919786312</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -674,14 +674,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>('DE', 'DK')</t>
+          <t>('RU', 'TR')</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>18425.94820709651</v>
+        <v>231563.3429361015</v>
       </c>
       <c r="D14" t="n">
-        <v>0.3708861076353018</v>
+        <v>0.6616123867276616</v>
       </c>
     </row>
     <row r="15">
@@ -692,7 +692,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>('FR', 'ES')</t>
+          <t>('CH', 'IT')</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -710,14 +710,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>('RO', 'BG')</t>
+          <t>('HU', 'HR')</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>22777.99741486265</v>
+        <v>22823.60655496021</v>
       </c>
       <c r="D16" t="n">
-        <v>0.07745016738378739</v>
+        <v>0.8078866785232456</v>
       </c>
     </row>
     <row r="17">
@@ -728,14 +728,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>('BG', 'MK')</t>
+          <t>('FR', 'CH')</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3174.72765343728</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0.3176728992702683</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -746,14 +746,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>('RU', 'DE')</t>
+          <t>('DE', 'FR')</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>513190</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -764,14 +764,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>('BY', 'PL')</t>
+          <t>('CZ', 'SK')</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>265850.1435398231</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0.6051986353496894</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -782,7 +782,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>('ES', 'FR')</t>
+          <t>('AT', 'HU')</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -800,14 +800,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>('NO', 'DE')</t>
+          <t>('TR', 'EL')</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>300492.8996512968</v>
+        <v>69066.54789252667</v>
       </c>
       <c r="D21" t="n">
-        <v>0.6601990523037137</v>
+        <v>0.4790466300851511</v>
       </c>
     </row>
     <row r="22">
@@ -818,14 +818,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>('TR', 'EL')</t>
+          <t>('CZ', 'PL')</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>69066.54789252667</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>0.4790466300851511</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -836,14 +836,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>('CH', 'DE')</t>
+          <t>('LV', 'LT')</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>23061.92868</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>0.9705586212991605</v>
       </c>
     </row>
     <row r="24">
@@ -854,14 +854,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>('BG', 'RS')</t>
+          <t>('TN', 'IT')</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>340797.7711173497</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>0.8203958559082485</v>
       </c>
     </row>
     <row r="25">
@@ -872,14 +872,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>('CZ', 'PL')</t>
+          <t>('BG', 'MK')</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>3174.72765343728</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>0.3176728992702683</v>
       </c>
     </row>
     <row r="26">
@@ -890,7 +890,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>('IT', 'SI')</t>
+          <t>('BE', 'FR')</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>('AL', 'IT')</t>
+          <t>('RO', 'UA')</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -926,14 +926,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>('NO', 'BE')</t>
+          <t>('BY', 'LT')</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>167754</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -944,14 +944,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>('PL', 'DE')</t>
+          <t>('NO', 'UK')</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>114691.6019731564</v>
+        <v>425847.6239331732</v>
       </c>
       <c r="D29" t="n">
-        <v>0.3372945116463543</v>
+        <v>0.8298049921728272</v>
       </c>
     </row>
     <row r="30">
@@ -962,14 +962,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>('NL', 'BE')</t>
+          <t>('MD', 'UA')</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>5319.754029749992</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>0.01043134023379438</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -980,7 +980,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>('CZ', 'SK')</t>
+          <t>('DE', 'PL')</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -998,14 +998,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>('BE', 'UK')</t>
+          <t>('EL', 'AL')</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>7162.06929252667</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>0.04028353038546089</v>
       </c>
     </row>
     <row r="33">
@@ -1016,14 +1016,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>('AT', 'IT')</t>
+          <t>('DK', 'DE')</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>78271.18871345268</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1864709677509296</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>('RO', 'MD')</t>
+          <t>('LU', 'BE')</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>('UK', 'NL')</t>
+          <t>('RS', 'HU')</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1070,14 +1070,14 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>('HR', 'HU')</t>
+          <t>('RU', 'DE')</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>513190</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>('FR', 'BE')</t>
+          <t>('DE', 'LU')</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>('ES', 'PT')</t>
+          <t>('RO', 'HU')</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>('DE', 'NL')</t>
+          <t>('BG', 'EL')</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>('AT', 'HU')</t>
+          <t>('SI', 'HR')</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>('RS', 'HU')</t>
+          <t>('SK', 'UA')</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1178,14 +1178,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>('RU', 'FI')</t>
+          <t>('ES', 'FR')</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>24443.12877777778</v>
+        <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>0.3043976186522763</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1196,14 +1196,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>('BY', 'LT')</t>
+          <t>('TR', 'BG')</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>8400.471468574746</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>0.03995449946159457</v>
       </c>
     </row>
     <row r="44">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>('SI', 'IT')</t>
+          <t>('EL', 'BG')</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1232,14 +1232,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>('BG', 'TR')</t>
+          <t>('BE', 'LU')</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>7059.178429749999</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>0.4607715707201311</v>
       </c>
     </row>
     <row r="46">
@@ -1250,14 +1250,14 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>('SK', 'AT')</t>
+          <t>('HR', 'SI')</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>85370.54174030092</v>
+        <v>2810.5</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1489377834812192</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1268,14 +1268,14 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>('BG', 'EL')</t>
+          <t>('AT', 'SI')</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>5492.305820583826</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>0.1337547840629242</v>
       </c>
     </row>
     <row r="48">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>('LV', 'RU')</t>
+          <t>('SK', 'HU')</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>('MD', 'UA')</t>
+          <t>('IT', 'AT')</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1322,14 +1322,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>('EL', 'BG')</t>
+          <t>('UA', 'SK')</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>211933.4410297454</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>0.2597010307116271</v>
       </c>
     </row>
     <row r="51">
@@ -1340,14 +1340,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>('BG', 'RO')</t>
+          <t>('DE', 'AT')</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>74142.4223062457</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>0.590068567215207</v>
       </c>
     </row>
     <row r="52">
@@ -1358,14 +1358,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>('UK', 'IE')</t>
+          <t>('NL', 'UK')</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>32030.28155817336</v>
+        <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2279329767527014</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1376,14 +1376,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>('BE', 'LU')</t>
+          <t>('UA', 'HU')</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>7059.178429749999</v>
+        <v>127297.4568654211</v>
       </c>
       <c r="D53" t="n">
-        <v>0.4607715707201311</v>
+        <v>0.6764161283857143</v>
       </c>
     </row>
     <row r="54">
@@ -1394,14 +1394,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>('NO', 'UK')</t>
+          <t>('NO', 'NL')</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>425847.6239331732</v>
+        <v>123813.4545419723</v>
       </c>
       <c r="D54" t="n">
-        <v>0.8298049921728272</v>
+        <v>0.3520287919786312</v>
       </c>
     </row>
     <row r="55">
@@ -1412,14 +1412,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>('LV', 'EE')</t>
+          <t>('RU', 'FI')</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>24443.12877777778</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>0.3043976186522763</v>
       </c>
     </row>
     <row r="56">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>('NL', 'UK')</t>
+          <t>('UA', 'PL')</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1448,14 +1448,14 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>('NO', 'FR')</t>
+          <t>('LT', 'RU')</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>73914.84975675003</v>
+        <v>0</v>
       </c>
       <c r="D57" t="n">
-        <v>0.3562118516969677</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>('DE', 'BE')</t>
+          <t>('PT', 'ES')</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1484,14 +1484,14 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>('RS', 'BA')</t>
+          <t>('DK', 'SE')</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>6562.7</v>
+        <v>9681.33725</v>
       </c>
       <c r="D59" t="n">
-        <v>1</v>
+        <v>0.6469319913130639</v>
       </c>
     </row>
     <row r="60">
@@ -1502,14 +1502,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>('RU', 'BY')</t>
+          <t>('BG', 'RS')</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>439277.4999999999</v>
+        <v>0</v>
       </c>
       <c r="D60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>('CH', 'FR')</t>
+          <t>('RS', 'BG')</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -1538,14 +1538,14 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>('HU', 'RS')</t>
+          <t>('RO', 'BG')</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>21350.96169934978</v>
+        <v>22777.99741486253</v>
       </c>
       <c r="D62" t="n">
-        <v>0.4119421512512016</v>
+        <v>0.07745016738378699</v>
       </c>
     </row>
     <row r="63">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>('MA', 'ES')</t>
+          <t>('LV', 'RU')</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>('CH', 'IT')</t>
+          <t>('UK', 'NL')</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>('AT', 'SK')</t>
+          <t>('AT', 'DE')</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>('LT', 'RU')</t>
+          <t>('CZ', 'DE')</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>('RS', 'BG')</t>
+          <t>('HU', 'SK')</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>('LY', 'IT')</t>
+          <t>('RU', 'UA')</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>48847.1869468165</v>
+        <v>486910</v>
       </c>
       <c r="D68" t="n">
-        <v>0.2812692506165045</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>('PT', 'ES')</t>
+          <t>('BE', 'NL')</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -1682,14 +1682,14 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>('DK', 'SE')</t>
+          <t>('BG', 'RO')</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>9681.33725</v>
+        <v>0</v>
       </c>
       <c r="D70" t="n">
-        <v>0.6469319913130639</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -1700,14 +1700,14 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>('CZ', 'DE')</t>
+          <t>('NO', 'DE')</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0</v>
+        <v>300492.8996512968</v>
       </c>
       <c r="D71" t="n">
-        <v>0</v>
+        <v>0.6601990523037137</v>
       </c>
     </row>
     <row r="72">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>('SK', 'UA')</t>
+          <t>('BE', 'UK')</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -1736,14 +1736,14 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>('EL', 'AL')</t>
+          <t>('DZ', 'MA')</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>7162.06929252667</v>
+        <v>7001.781042743663</v>
       </c>
       <c r="D73" t="n">
-        <v>0.04028353038546089</v>
+        <v>0.0569058491870114</v>
       </c>
     </row>
     <row r="74">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>('AT', 'DE')</t>
+          <t>('ES', 'PT')</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -1772,14 +1772,14 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>('RU', 'UA')</t>
+          <t>('MD', 'RO')</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>486910</v>
+        <v>0</v>
       </c>
       <c r="D75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>('EE', 'FI')</t>
+          <t>('LV', 'EE')</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -1808,14 +1808,14 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>('UA', 'PL')</t>
+          <t>('SK', 'AT')</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0</v>
+        <v>85370.54174030101</v>
       </c>
       <c r="D77" t="n">
-        <v>0</v>
+        <v>0.1489377834812194</v>
       </c>
     </row>
     <row r="78">
@@ -1826,14 +1826,14 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>('FI', 'EE')</t>
+          <t>('DE', 'DK')</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4201.588500000001</v>
+        <v>18425.94820709651</v>
       </c>
       <c r="D78" t="n">
-        <v>0.3509271885270984</v>
+        <v>0.3708861076353018</v>
       </c>
     </row>
     <row r="79">
@@ -1844,14 +1844,14 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>('SK', 'CZ')</t>
+          <t>('CH', 'DE')</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>80761.751</v>
+        <v>0</v>
       </c>
       <c r="D79" t="n">
-        <v>0.4835338095124054</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -1862,14 +1862,14 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>('IT', 'AT')</t>
+          <t>('LY', 'IT')</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0</v>
+        <v>48847.1869468165</v>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
+        <v>0.2812692506165045</v>
       </c>
     </row>
     <row r="81">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>('RO', 'UA')</t>
+          <t>('BG', 'TR')</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>('HU', 'SK')</t>
+          <t>('IT', 'SI')</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -1916,14 +1916,14 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>('HR', 'SI')</t>
+          <t>('BE', 'DE')</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2810.5</v>
+        <v>0</v>
       </c>
       <c r="D83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>('FR', 'CH')</t>
+          <t>('RO', 'MD')</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -1952,14 +1952,14 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>('BE', 'DE')</t>
+          <t>('SK', 'CZ')</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0</v>
+        <v>80761.751</v>
       </c>
       <c r="D85" t="n">
-        <v>0</v>
+        <v>0.4835338095124054</v>
       </c>
     </row>
     <row r="86">
@@ -1970,14 +1970,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>('TN', 'IT')</t>
+          <t>('RU', 'LV')</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>339332.2711173499</v>
+        <v>33546.970555</v>
       </c>
       <c r="D86" t="n">
-        <v>0.8168679862191611</v>
+        <v>0.5470804069634703</v>
       </c>
     </row>
     <row r="87">
@@ -1988,14 +1988,14 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>('UK', 'BE')</t>
+          <t>('BY', 'PL')</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>0</v>
+        <v>265850.1435398231</v>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
+        <v>0.6051986353496894</v>
       </c>
     </row>
     <row r="88">
@@ -2006,14 +2006,14 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>('DZ', 'MA')</t>
+          <t>('NO', 'BE')</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>7001.781042743663</v>
+        <v>167754</v>
       </c>
       <c r="D88" t="n">
-        <v>0.0569058491870114</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -2024,14 +2024,14 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>('AT', 'SI')</t>
+          <t>('DE', 'NL')</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>5492.305820583826</v>
+        <v>0</v>
       </c>
       <c r="D89" t="n">
-        <v>0.1337547840629242</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -2042,14 +2042,14 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>('UA', 'SK')</t>
+          <t>('EE', 'FI')</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>211933.4410297454</v>
+        <v>0</v>
       </c>
       <c r="D90" t="n">
-        <v>0.259701030711627</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -2060,14 +2060,14 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>('DE', 'CZ')</t>
+          <t>('UA', 'RO')</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>0</v>
+        <v>44717.04995347363</v>
       </c>
       <c r="D91" t="n">
-        <v>0</v>
+        <v>0.6077007223509681</v>
       </c>
     </row>
     <row r="92">
@@ -2078,14 +2078,14 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>('DE', 'AT')</t>
+          <t>('UK', 'IE')</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>74142.42230624572</v>
+        <v>32030.28155817336</v>
       </c>
       <c r="D92" t="n">
-        <v>0.5900685672152071</v>
+        <v>0.2279329767527014</v>
       </c>
     </row>
     <row r="93">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>('IT', 'CH')</t>
+          <t>('DE', 'CZ')</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>('DE', 'FR')</t>
+          <t>('IT', 'CH')</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>('BY', 'UA')</t>
+          <t>('NL', 'DE')</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -2150,14 +2150,14 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>('HU', 'RO')</t>
+          <t>('HU', 'RS')</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>0</v>
+        <v>21350.96169934978</v>
       </c>
       <c r="D96" t="n">
-        <v>0</v>
+        <v>0.4119421512512016</v>
       </c>
     </row>
     <row r="97">
@@ -2168,14 +2168,14 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>('TR', 'BG')</t>
+          <t>('UK', 'BE')</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>8400.471468574629</v>
+        <v>0</v>
       </c>
       <c r="D97" t="n">
-        <v>0.03995449946159401</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -2186,14 +2186,14 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>('SK', 'HU')</t>
+          <t>('DE', 'CH')</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>0</v>
+        <v>32384.83611111111</v>
       </c>
       <c r="D98" t="n">
-        <v>0</v>
+        <v>0.270504812154286</v>
       </c>
     </row>
     <row r="99">
@@ -2204,14 +2204,14 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>('UA', 'HU')</t>
+          <t>('NO', 'FR')</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>127297.4568654211</v>
+        <v>73914.84975675003</v>
       </c>
       <c r="D99" t="n">
-        <v>0.6764161283857143</v>
+        <v>0.3562118516969677</v>
       </c>
     </row>
     <row r="100">
@@ -2222,14 +2222,14 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>('LV', 'LT')</t>
+          <t>('RU', 'BY')</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>23061.92868</v>
+        <v>439277.4999999999</v>
       </c>
       <c r="D100" t="n">
-        <v>0.9705586212991605</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>('LU', 'BE')</t>
+          <t>('MA', 'ES')</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -2258,14 +2258,14 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>('DE', 'CH')</t>
+          <t>('AT', 'SK')</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>32384.83611111111</v>
+        <v>0</v>
       </c>
       <c r="D102" t="n">
-        <v>0.270504812154286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -2276,14 +2276,14 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>('RU', 'TR')</t>
+          <t>('UA', 'MD')</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>231563.3429361014</v>
+        <v>6993.868709865174</v>
       </c>
       <c r="D103" t="n">
-        <v>0.6616123867276613</v>
+        <v>0.07500684468945812</v>
       </c>
     </row>
     <row r="104">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>('BE', 'NL')</t>
+          <t>('SI', 'IT')</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -2312,14 +2312,14 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>('UA', 'RO')</t>
+          <t>('HR', 'HU')</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>44717.04995347375</v>
+        <v>0</v>
       </c>
       <c r="D105" t="n">
-        <v>0.6077007223509696</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>('SI', 'HR')</t>
+          <t>('CH', 'FR')</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -2348,14 +2348,14 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>('HU', 'HR')</t>
+          <t>('HU', 'RO')</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>22823.60655496021</v>
+        <v>0</v>
       </c>
       <c r="D107" t="n">
-        <v>0.8078866785232456</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>('RO', 'HU')</t>
+          <t>('BY', 'UA')</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -2384,14 +2384,14 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>('NL', 'DE')</t>
+          <t>('DZ', 'TN')</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>0</v>
+        <v>357313.498390077</v>
       </c>
       <c r="D109" t="n">
-        <v>0</v>
+        <v>0.8601538454262924</v>
       </c>
     </row>
     <row r="110">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>('LT_LNG_imp', 'LT')</t>
+          <t>('NL_LNG_imp', 'NL')</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -2420,14 +2420,14 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>('BE_LNG_imp', 'BE')</t>
+          <t>('ES_LNG_imp', 'ES')</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>0</v>
+        <v>309306.8176735208</v>
       </c>
       <c r="D111" t="n">
-        <v>0</v>
+        <v>0.5267693006938637</v>
       </c>
     </row>
     <row r="112">
@@ -2438,14 +2438,14 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>('FR_LNG_imp', 'FR')</t>
+          <t>('PL_LNG_imp', 'PL')</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>322409.9999999999</v>
+        <v>0</v>
       </c>
       <c r="D112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>('TR_LNG_imp', 'TR')</t>
+          <t>('HR_LNG_imp', 'HR')</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -2478,7 +2478,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>155831.5</v>
+        <v>154366</v>
       </c>
       <c r="D114" t="n">
         <v>1</v>
@@ -2492,14 +2492,14 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>('HR_LNG_imp', 'HR')</t>
+          <t>('FR_LNG_imp', 'FR')</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>0</v>
+        <v>322409.9999999999</v>
       </c>
       <c r="D115" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -2510,14 +2510,14 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>('PT_LNG_imp', 'PT')</t>
+          <t>('UK_LNG_imp', 'UK')</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>58978.16446262326</v>
+        <v>0</v>
       </c>
       <c r="D116" t="n">
-        <v>0.7942973180873681</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>('PL_LNG_imp', 'PL')</t>
+          <t>('EL_LNG_imp', 'EL')</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>('EL_LNG_imp', 'EL')</t>
+          <t>('BE_LNG_imp', 'BE')</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>('UK_LNG_imp', 'UK')</t>
+          <t>('TR_LNG_imp', 'TR')</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -2582,14 +2582,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>('ES_LNG_imp', 'ES')</t>
+          <t>('PT_LNG_imp', 'PT')</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>307841.3176735209</v>
+        <v>58978.16446262326</v>
       </c>
       <c r="D120" t="n">
-        <v>0.4695802529314639</v>
+        <v>0.8269396736252052</v>
       </c>
     </row>
     <row r="121">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>('NL_LNG_imp', 'NL')</t>
+          <t>('LT_LNG_imp', 'LT')</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -2618,14 +2618,14 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>('EG_LNG_imp', 'EG')</t>
+          <t>('JS_LNG_imp', 'JS')</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>0</v>
+        <v>1579465.226022091</v>
       </c>
       <c r="D122" t="n">
-        <v>0</v>
+        <v>0.1579465383968629</v>
       </c>
     </row>
     <row r="123">
@@ -2654,14 +2654,14 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>('AS_LNG_imp', 'AS')</t>
+          <t>('CN_LNG_imp', 'CN')</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>339902.243945254</v>
+        <v>766145.0242350446</v>
       </c>
       <c r="D124" t="n">
-        <v>0.03399022779354818</v>
+        <v>0.07661451008495547</v>
       </c>
     </row>
     <row r="125">
@@ -2672,14 +2672,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>('IN_LNG_imp', 'IN')</t>
+          <t>('AF_LNG_imp', 'AF')</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>357577.0638860887</v>
+        <v>0</v>
       </c>
       <c r="D125" t="n">
-        <v>0.03575770996437987</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126">
@@ -2690,14 +2690,14 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>('CN_LNG_imp', 'CN')</t>
+          <t>('AS_LNG_imp', 'AS')</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>766145.0242350446</v>
+        <v>339902.243945254</v>
       </c>
       <c r="D126" t="n">
-        <v>0.07661451008495547</v>
+        <v>0.03399022779354818</v>
       </c>
     </row>
     <row r="127">
@@ -2708,14 +2708,14 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>('JS_LNG_imp', 'JS')</t>
+          <t>('IN_LNG_imp', 'IN')</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1579465.226022091</v>
+        <v>357577.0638860887</v>
       </c>
       <c r="D127" t="n">
-        <v>0.1579465383968629</v>
+        <v>0.03575770996437987</v>
       </c>
     </row>
     <row r="128">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>('AF_LNG_imp', 'AF')</t>
+          <t>('EG_LNG_imp', 'EG')</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -2762,14 +2762,14 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>('ME', 'ME_LNG_exp')</t>
+          <t>('AU', 'AU_LNG_exp')</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>0</v>
+        <v>999349.7079159727</v>
       </c>
       <c r="D130" t="n">
-        <v>0</v>
+        <v>0.09993498078509534</v>
       </c>
     </row>
     <row r="131">
@@ -2780,14 +2780,14 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>('AU', 'AU_LNG_exp')</t>
+          <t>('ME', 'ME_LNG_exp')</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>999349.7079159727</v>
+        <v>0</v>
       </c>
       <c r="D131" t="n">
-        <v>0.09993498078509534</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
@@ -2798,14 +2798,14 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>('QA', 'QA_LNG_exp')</t>
+          <t>('EG', 'EG_LNG_exp')</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1123959.165391228</v>
+        <v>1536.335261238157</v>
       </c>
       <c r="D132" t="n">
-        <v>0.1123959277787156</v>
+        <v>0.0001536335414871698</v>
       </c>
     </row>
     <row r="133">
@@ -2816,14 +2816,14 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>('IM', 'IM_LNG_exp')</t>
+          <t>('USA', 'USA_LNG_exp')</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>504093.1518337181</v>
+        <v>819373.0123329933</v>
       </c>
       <c r="D133" t="n">
-        <v>0.05040932022430383</v>
+        <v>0.08193730942703027</v>
       </c>
     </row>
     <row r="134">
@@ -2852,14 +2852,14 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>('USA', 'USA_LNG_exp')</t>
+          <t>('IM', 'IM_LNG_exp')</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>819373.0123329933</v>
+        <v>504093.1518337181</v>
       </c>
       <c r="D135" t="n">
-        <v>0.08193730942703027</v>
+        <v>0.05040932022430383</v>
       </c>
     </row>
     <row r="136">
@@ -2870,14 +2870,14 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>('TT', 'TT_LNG_exp')</t>
+          <t>('QA', 'QA_LNG_exp')</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>139511.8579414433</v>
+        <v>1123959.165391228</v>
       </c>
       <c r="D136" t="n">
-        <v>0.01395118718926305</v>
+        <v>0.1123959277787156</v>
       </c>
     </row>
     <row r="137">
@@ -2888,14 +2888,14 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>('EG', 'EG_LNG_exp')</t>
+          <t>('TT', 'TT_LNG_exp')</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1536.335261238157</v>
+        <v>139511.8579414433</v>
       </c>
       <c r="D137" t="n">
-        <v>0.0001536335414871698</v>
+        <v>0.01395118718926305</v>
       </c>
     </row>
     <row r="138">
@@ -2906,14 +2906,14 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>('RU', 'CN')</t>
+          <t>('ME', 'AF')</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>371260</v>
+        <v>0</v>
       </c>
       <c r="D138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -2924,14 +2924,14 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>('USA', 'CM')</t>
+          <t>('ME', 'CR')</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>62499.4175759519</v>
+        <v>0</v>
       </c>
       <c r="D139" t="n">
-        <v>0.01279414894082946</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>('ME', 'QA')</t>
+          <t>('AS', 'CN')</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -2960,14 +2960,14 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>('ME', 'CR')</t>
+          <t>('RU', 'CN')</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>0</v>
+        <v>371260</v>
       </c>
       <c r="D141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -2978,14 +2978,14 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>('AS', 'CN')</t>
+          <t>('CR', 'CN')</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>0</v>
+        <v>255875.5104257212</v>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>0.727497755105542</v>
       </c>
     </row>
     <row r="143">
@@ -3014,14 +3014,14 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>('CR', 'TR')</t>
+          <t>('RU', 'CR')</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>293099.9999999999</v>
+        <v>0</v>
       </c>
       <c r="D144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
@@ -3032,14 +3032,14 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>('CR', 'CN')</t>
+          <t>('USA', 'CM')</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>255875.5104257212</v>
+        <v>62499.4175759519</v>
       </c>
       <c r="D145" t="n">
-        <v>0.727497755105542</v>
+        <v>0.01279414894082946</v>
       </c>
     </row>
     <row r="146">
@@ -3050,14 +3050,14 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>('ME', 'AF')</t>
+          <t>('CR', 'TR')</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>0</v>
+        <v>293099.9999999999</v>
       </c>
       <c r="D146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>('RU', 'CR')</t>
+          <t>('ME', 'QA')</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -3122,7 +3122,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'AF_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'AF_LNG_imp')</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'AF_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -3230,14 +3230,14 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1536.335261238157</v>
+        <v>233204.6836809279</v>
       </c>
       <c r="D156" t="n">
-        <v>0.0001536335414871698</v>
+        <v>0.02332047070013986</v>
       </c>
     </row>
     <row r="157">
@@ -3248,14 +3248,14 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>0</v>
+        <v>357577.0638860887</v>
       </c>
       <c r="D157" t="n">
-        <v>0</v>
+        <v>0.03575770996437987</v>
       </c>
     </row>
     <row r="158">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'EG_LNG_imp')</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -3284,14 +3284,14 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'EG_LNG_imp')</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>233204.6836809279</v>
+        <v>0</v>
       </c>
       <c r="D159" t="n">
-        <v>0.02332047070013986</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -3338,7 +3338,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'ES_LNG_imp')</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'AS_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'AF_LNG_imp')</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -3428,14 +3428,14 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>357577.0638860887</v>
+        <v>0</v>
       </c>
       <c r="D167" t="n">
-        <v>0.03575770996437987</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'EG_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'AF_LNG_imp')</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -3608,14 +3608,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'ES_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>19661.40057959002</v>
+        <v>0</v>
       </c>
       <c r="D177" t="n">
-        <v>0.001966140254573027</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'ES_LNG_imp')</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -3680,14 +3680,14 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>0</v>
+        <v>766145.0242350447</v>
       </c>
       <c r="D181" t="n">
-        <v>0</v>
+        <v>0.07661451008495548</v>
       </c>
     </row>
     <row r="182">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -3734,14 +3734,14 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'ES_LNG_imp')</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>415687.5329475594</v>
+        <v>0</v>
       </c>
       <c r="D184" t="n">
-        <v>0.04156875745163169</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185">
@@ -3752,14 +3752,14 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'AS_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'AS_LNG_imp')</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>339902.243945254</v>
+        <v>0</v>
       </c>
       <c r="D185" t="n">
-        <v>0.03399022779354818</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -3878,7 +3878,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'AF_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -3932,14 +3932,14 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>0</v>
+        <v>426479.8575598855</v>
       </c>
       <c r="D195" t="n">
-        <v>0</v>
+        <v>0.04264799002078755</v>
       </c>
     </row>
     <row r="196">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -4004,7 +4004,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'AS_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'AS_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -4094,14 +4094,14 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'ES_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>81275.47938543411</v>
+        <v>0</v>
       </c>
       <c r="D204" t="n">
-        <v>0.008127548751298286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'AS_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -4148,14 +4148,14 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'ES_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>206904.4377084968</v>
+        <v>0</v>
       </c>
       <c r="D207" t="n">
-        <v>0.02069044583989427</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'AS_LNG_imp')</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -4238,7 +4238,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'EG_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'ES_LNG_imp')</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -4364,14 +4364,14 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>504093.1518337181</v>
+        <v>0</v>
       </c>
       <c r="D219" t="n">
-        <v>0.05040932022430383</v>
+        <v>0</v>
       </c>
     </row>
     <row r="220">
@@ -4382,14 +4382,14 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>0</v>
+        <v>58978.16446262326</v>
       </c>
       <c r="D220" t="n">
-        <v>0</v>
+        <v>0.005897817036044029</v>
       </c>
     </row>
     <row r="221">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -4418,14 +4418,14 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'ES_LNG_imp')</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>0</v>
+        <v>19661.40057959002</v>
       </c>
       <c r="D222" t="n">
-        <v>0</v>
+        <v>0.001966140254573027</v>
       </c>
     </row>
     <row r="223">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'EG_LNG_imp')</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'AF_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -4490,14 +4490,14 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>0</v>
+        <v>1536.335261238157</v>
       </c>
       <c r="D226" t="n">
-        <v>0</v>
+        <v>0.0001536335414871698</v>
       </c>
     </row>
     <row r="227">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'ES_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'AS_LNG_imp')</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -4616,7 +4616,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'EG_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -4652,7 +4652,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'AF_LNG_imp')</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -4688,14 +4688,14 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>0</v>
+        <v>415687.5329475596</v>
       </c>
       <c r="D237" t="n">
-        <v>0</v>
+        <v>0.04156875745163171</v>
       </c>
     </row>
     <row r="238">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -4724,7 +4724,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -4778,14 +4778,14 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0</v>
+        <v>152829.6647387618</v>
       </c>
       <c r="D242" t="n">
-        <v>0</v>
+        <v>0.01528296800217298</v>
       </c>
     </row>
     <row r="243">
@@ -4796,14 +4796,14 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'ES_LNG_imp')</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0</v>
+        <v>208369.9377084968</v>
       </c>
       <c r="D243" t="n">
-        <v>0</v>
+        <v>0.02083699585454927</v>
       </c>
     </row>
     <row r="244">
@@ -4814,14 +4814,14 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'ES_LNG_imp')</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>426479.8575598855</v>
+        <v>0</v>
       </c>
       <c r="D244" t="n">
-        <v>0.04264799002078755</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'AS_LNG_imp')</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'ES_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -4868,7 +4868,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'AF_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -4904,14 +4904,14 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>58978.16446262326</v>
+        <v>0</v>
       </c>
       <c r="D249" t="n">
-        <v>0.005897817036044029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -4940,14 +4940,14 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'AF_LNG_imp')</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>60872.29289923003</v>
+        <v>0</v>
       </c>
       <c r="D251" t="n">
-        <v>0.006087229898645993</v>
+        <v>0</v>
       </c>
     </row>
     <row r="252">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -5048,7 +5048,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'EG_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'AF_LNG_imp')</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -5084,14 +5084,14 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'AF_LNG_imp')</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>154295.1647387618</v>
+        <v>0</v>
       </c>
       <c r="D259" t="n">
-        <v>0.01542951801682799</v>
+        <v>0</v>
       </c>
     </row>
     <row r="260">
@@ -5102,14 +5102,14 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'AS_LNG_imp')</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>0</v>
+        <v>339902.243945254</v>
       </c>
       <c r="D260" t="n">
-        <v>0</v>
+        <v>0.03399022779354818</v>
       </c>
     </row>
     <row r="261">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'ES_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -5156,14 +5156,14 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'EG_LNG_imp')</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>766145.0242350447</v>
+        <v>0</v>
       </c>
       <c r="D263" t="n">
-        <v>0.07661451008495548</v>
+        <v>0</v>
       </c>
     </row>
     <row r="264">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -5228,14 +5228,14 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>322409.9999999999</v>
+        <v>0</v>
       </c>
       <c r="D267" t="n">
-        <v>0.03224100322410031</v>
+        <v>0</v>
       </c>
     </row>
     <row r="268">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'AS_LNG_imp')</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'AF_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'ES_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -5390,14 +5390,14 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>0</v>
+        <v>504093.1518337181</v>
       </c>
       <c r="D276" t="n">
-        <v>0</v>
+        <v>0.05040932022430383</v>
       </c>
     </row>
     <row r="277">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'EG_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'EG_LNG_imp')</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -5426,14 +5426,14 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'EG_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C278" t="n">
-        <v>0</v>
+        <v>60872.29289923003</v>
       </c>
       <c r="D278" t="n">
-        <v>0</v>
+        <v>0.006087229898645993</v>
       </c>
     </row>
     <row r="279">
@@ -5444,7 +5444,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'EG_LNG_imp')</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'ES_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'JS_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'AS_LNG_imp')</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'PL_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -5570,7 +5570,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'AS_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -5588,7 +5588,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'AF_LNG_imp')</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -5606,14 +5606,14 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'AS_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'FR_LNG_imp')</t>
         </is>
       </c>
       <c r="C288" t="n">
-        <v>0</v>
+        <v>322409.9999999999</v>
       </c>
       <c r="D288" t="n">
-        <v>0</v>
+        <v>0.03224100322410031</v>
       </c>
     </row>
     <row r="289">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'AF_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'PL_LNG_imp')</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'JS_LNG_imp')</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'IN_LNG_imp')</t>
+          <t>('IM_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -5750,7 +5750,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'EL_LNG_imp')</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'TR_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'UK_LNG_imp')</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'HR_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'IT_LNG_imp')</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -5804,14 +5804,14 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'EG_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'ES_LNG_imp')</t>
         </is>
       </c>
       <c r="C299" t="n">
-        <v>0</v>
+        <v>81275.479385434</v>
       </c>
       <c r="D299" t="n">
-        <v>0</v>
+        <v>0.008127548751298275</v>
       </c>
     </row>
     <row r="300">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'AS_LNG_imp')</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>('TT_LNG_exp', 'LT_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'CN_LNG_imp')</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'HR_LNG_imp')</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'EG_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>('RU_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'BE_LNG_imp')</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'EL_LNG_imp')</t>
+          <t>('AU_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -5930,7 +5930,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'BE_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>('AU_LNG_exp', 'AS_LNG_imp')</t>
+          <t>('RU_LNG_exp', 'PT_LNG_imp')</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>('IM_LNG_exp', 'CN_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'SA_LNG_imp')</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -5984,7 +5984,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('QA_LNG_exp', 'EG_LNG_imp')</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>('QA_LNG_exp', 'IT_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'FR_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -6038,7 +6038,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'NL_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'NL_LNG_imp')</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>('USA_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('EG_LNG_exp', 'TR_LNG_imp')</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -6074,7 +6074,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>('AF_LNG_exp', 'UK_LNG_imp')</t>
+          <t>('TT_LNG_exp', 'EG_LNG_imp')</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -6092,7 +6092,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'PT_LNG_imp')</t>
+          <t>('USA_LNG_exp', 'LT_LNG_imp')</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>('EG_LNG_exp', 'AF_LNG_imp')</t>
+          <t>('AF_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>('ME_LNG_exp', 'SA_LNG_imp')</t>
+          <t>('ME_LNG_exp', 'IN_LNG_imp')</t>
         </is>
       </c>
       <c r="C317" t="n">

</xml_diff>